<commit_message>
Sync with current pipeline: form-filler agent, /outcome, model routing, six-part cover letters, still-open check, context limits, rules 14-21
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/applications/applied.xlsx
+++ b/applications/applied.xlsx
@@ -441,7 +441,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:M1"/>
+  <dimension ref="A1:N1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -457,6 +457,7 @@
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="50" customWidth="1" min="12" max="12"/>
     <col width="45" customWidth="1" min="13" max="13"/>
+    <col width="40" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -525,9 +526,19 @@
           <t>Answers</t>
         </is>
       </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Rejection Reason</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:M1"/>
+  <dataValidations count="1">
+    <dataValidation sqref="A2:A500" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Application submitted,Rejected"</formula1>
+    </dataValidation>
+  </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>